<commit_message>
Robô: atualiza laudos.xlsx (20/10/2026 15:39)
</commit_message>
<xml_diff>
--- a/laudos.xlsx
+++ b/laudos.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Amostras" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alertas" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Resultados" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Amostras" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Matriz" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Alertas" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Log" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resultados'!$A$1:$W$68</definedName>
@@ -7706,7 +7706,7 @@
       </c>
       <c r="X2" s="3" t="inlineStr">
         <is>
-          <t>02_PROCESSADOS/2026/2026-09/2026-09-30_AB_GOIABAL_4293-2026.pdf</t>
+          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_GOIABAL_4293-2026.pdf</t>
         </is>
       </c>
       <c r="Y2" s="3" t="inlineStr">
@@ -7817,7 +7817,7 @@
       </c>
       <c r="X3" s="3" t="inlineStr">
         <is>
-          <t>02_PROCESSADOS/2026/2026-09/2026-09-30_AB_MONTANTE_4296-2026.pdf</t>
+          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_MONTANTE_4296-2026.pdf</t>
         </is>
       </c>
       <c r="Y3" s="3" t="inlineStr">
@@ -7928,7 +7928,7 @@
       </c>
       <c r="X4" s="3" t="inlineStr">
         <is>
-          <t>02_PROCESSADOS/2026/2026-09/2026-09-30_AB_JUSANTE_4294-2026.pdf</t>
+          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_JUSANTE_4294-2026.pdf</t>
         </is>
       </c>
       <c r="Y4" s="3" t="inlineStr">
@@ -8039,7 +8039,7 @@
       </c>
       <c r="X5" s="3" t="inlineStr">
         <is>
-          <t>02_PROCESSADOS/2026/2026-09/2026-09-30_AB_CAPTACAO_4295-2026.pdf</t>
+          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_CAPTACAO_4295-2026.pdf</t>
         </is>
       </c>
       <c r="Y5" s="3" t="inlineStr">
@@ -8154,7 +8154,7 @@
       </c>
       <c r="X6" s="3" t="inlineStr">
         <is>
-          <t>02_PROCESSADOS/2026/2026-09/2026-09-30_AB_SAIDA-DA-MINA_4291-2026.pdf</t>
+          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_SAIDA-DA-MINA_4291-2026.pdf</t>
         </is>
       </c>
       <c r="Y6" s="3" t="inlineStr">
@@ -8273,7 +8273,7 @@
       </c>
       <c r="X7" s="3" t="inlineStr">
         <is>
-          <t>02_PROCESSADOS/2026/2026-09/2026-09-30_AB_JUSANTE_4219-2026.pdf</t>
+          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_JUSANTE_4219-2026.pdf</t>
         </is>
       </c>
       <c r="Y7" s="3" t="inlineStr">
@@ -8384,7 +8384,7 @@
       </c>
       <c r="X8" s="3" t="inlineStr">
         <is>
-          <t>02_PROCESSADOS/2026/2026-09/2026-09-30_AR_LAGOA-01_4221-2026.pdf</t>
+          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AR_LAGOA-01_4221-2026.pdf</t>
         </is>
       </c>
       <c r="Y8" s="3" t="inlineStr">
@@ -8495,7 +8495,7 @@
       </c>
       <c r="X9" s="3" t="inlineStr">
         <is>
-          <t>02_PROCESSADOS/2026/2026-09/2026-09-30_AR_LAGOA-07_4220-2026.pdf</t>
+          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AR_LAGOA-07_4220-2026.pdf</t>
         </is>
       </c>
       <c r="Y9" s="3" t="inlineStr">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="X10" s="3" t="inlineStr">
         <is>
-          <t>02_PROCESSADOS/2026/2026-09/2026-09-30_AB_REPRESA-1_4218-2026.pdf</t>
+          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_REPRESA-1_4218-2026.pdf</t>
         </is>
       </c>
       <c r="Y10" s="3" t="inlineStr">
@@ -8725,7 +8725,7 @@
       </c>
       <c r="X11" s="3" t="inlineStr">
         <is>
-          <t>02_PROCESSADOS/2026/2026-09/2026-09-30_AB_REPRESA-1_4292-2026.pdf</t>
+          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_REPRESA-1_4292-2026.pdf</t>
         </is>
       </c>
       <c r="Y11" s="3" t="inlineStr">
@@ -10063,7 +10063,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 14:39:02</t>
+          <t>2026-10-20 14:48:36</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -10086,14 +10086,14 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>02_PROCESSADOS/2026/2026-09/2026-09-30_AB_MONTANTE_4296-2026.pdf</t>
+          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_MONTANTE_4296-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 14:39:02</t>
+          <t>2026-10-20 14:48:36</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -10116,14 +10116,14 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>02_PROCESSADOS/2026/2026-09/2026-09-30_AB_CAPTACAO_4295-2026.pdf</t>
+          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_CAPTACAO_4295-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 14:39:02</t>
+          <t>2026-10-20 14:48:36</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -10146,14 +10146,14 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>02_PROCESSADOS/2026/2026-09/2026-09-30_AB_JUSANTE_4294-2026.pdf</t>
+          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_JUSANTE_4294-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 14:39:02</t>
+          <t>2026-10-20 14:48:36</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -10176,14 +10176,14 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>02_PROCESSADOS/2026/2026-09/2026-09-30_AB_GOIABAL_4293-2026.pdf</t>
+          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_GOIABAL_4293-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 14:39:02</t>
+          <t>2026-10-20 14:48:36</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -10206,14 +10206,14 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>02_PROCESSADOS/2026/2026-09/2026-09-30_AB_REPRESA-1_4292-2026.pdf</t>
+          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_REPRESA-1_4292-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 14:39:02</t>
+          <t>2026-10-20 14:48:36</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -10236,14 +10236,14 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>02_PROCESSADOS/2026/2026-09/2026-09-30_AB_SAIDA-DA-MINA_4291-2026.pdf</t>
+          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_SAIDA-DA-MINA_4291-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 14:39:02</t>
+          <t>2026-10-20 14:48:36</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -10266,14 +10266,14 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>02_PROCESSADOS/2026/2026-09/2026-09-30_AR_LAGOA-01_4221-2026.pdf</t>
+          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AR_LAGOA-01_4221-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 14:39:02</t>
+          <t>2026-10-20 14:48:36</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -10296,14 +10296,14 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>02_PROCESSADOS/2026/2026-09/2026-09-30_AR_LAGOA-07_4220-2026.pdf</t>
+          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AR_LAGOA-07_4220-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 14:39:02</t>
+          <t>2026-10-20 14:48:36</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -10326,14 +10326,14 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>02_PROCESSADOS/2026/2026-09/2026-09-30_AB_JUSANTE_4219-2026.pdf</t>
+          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_JUSANTE_4219-2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 14:39:02</t>
+          <t>2026-10-20 14:48:36</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -10356,7 +10356,7 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>02_PROCESSADOS/2026/2026-09/2026-09-30_AB_REPRESA-1_4218-2026.pdf</t>
+          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_REPRESA-1_4218-2026.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Robô: atualiza laudos.xlsx (20/10/2026 16:19)
</commit_message>
<xml_diff>
--- a/laudos.xlsx
+++ b/laudos.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resultados'!$A$1:$W$68</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Amostras'!$A$1:$Y$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Alertas'!$A$1:$G$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Log'!$A$1:$F$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Log'!$A$1:$F$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -10017,11 +10017,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -10063,30 +10063,26 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>2026-10-20 14:48:36</t>
+          <t>2026-10-20 16:19:28</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>4296-1-2026_0.pdf</t>
+          <t>19813-2026 - 1-0.pdf</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Processado</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>4296-1/2026.0</t>
-        </is>
-      </c>
+          <t>ERRO</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n"/>
       <c r="E2" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_MONTANTE_4296-2026.pdf</t>
+          <t>Não parece um laudo Aqualit (texto 'Relatório de Análises' não encontrado). Pode ser um PDF escaneado ou de outro laboratório. — movido para 03_ERROS</t>
         </is>
       </c>
     </row>
@@ -10098,7 +10094,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>4295-1-2026_0.pdf</t>
+          <t>4296-1-2026_0.pdf</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -10108,15 +10104,15 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>4295-1/2026.0</t>
+          <t>4296-1/2026.0</t>
         </is>
       </c>
       <c r="E3" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_CAPTACAO_4295-2026.pdf</t>
+          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_MONTANTE_4296-2026.pdf</t>
         </is>
       </c>
     </row>
@@ -10128,7 +10124,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>4294-1-2026_0.pdf</t>
+          <t>4295-1-2026_0.pdf</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -10138,15 +10134,15 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>4294-1/2026.0</t>
+          <t>4295-1/2026.0</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_JUSANTE_4294-2026.pdf</t>
+          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_CAPTACAO_4295-2026.pdf</t>
         </is>
       </c>
     </row>
@@ -10158,7 +10154,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>4293-1-2026_0.pdf</t>
+          <t>4294-1-2026_0.pdf</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -10168,7 +10164,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>4293-1/2026.0</t>
+          <t>4294-1/2026.0</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
@@ -10176,7 +10172,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_GOIABAL_4293-2026.pdf</t>
+          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_JUSANTE_4294-2026.pdf</t>
         </is>
       </c>
     </row>
@@ -10188,7 +10184,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>4292-1-2026_0.pdf</t>
+          <t>4293-1-2026_0.pdf</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -10198,7 +10194,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>4292-1/2026.0</t>
+          <t>4293-1/2026.0</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
@@ -10206,7 +10202,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_REPRESA-1_4292-2026.pdf</t>
+          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_GOIABAL_4293-2026.pdf</t>
         </is>
       </c>
     </row>
@@ -10218,7 +10214,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>4291-1-2026_0.pdf</t>
+          <t>4292-1-2026_0.pdf</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -10228,7 +10224,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>4291-1/2026.0</t>
+          <t>4292-1/2026.0</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
@@ -10236,7 +10232,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_SAIDA-DA-MINA_4291-2026.pdf</t>
+          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_REPRESA-1_4292-2026.pdf</t>
         </is>
       </c>
     </row>
@@ -10248,7 +10244,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>4221-1-2026_0.pdf</t>
+          <t>4291-1-2026_0.pdf</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -10258,15 +10254,15 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>4221-1/2026.0</t>
+          <t>4291-1/2026.0</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AR_LAGOA-01_4221-2026.pdf</t>
+          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_SAIDA-DA-MINA_4291-2026.pdf</t>
         </is>
       </c>
     </row>
@@ -10278,7 +10274,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>4220-1-2026_0.pdf</t>
+          <t>4221-1-2026_0.pdf</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -10288,7 +10284,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>4220-1/2026.0</t>
+          <t>4221-1/2026.0</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -10296,7 +10292,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AR_LAGOA-07_4220-2026.pdf</t>
+          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AR_LAGOA-01_4221-2026.pdf</t>
         </is>
       </c>
     </row>
@@ -10308,7 +10304,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>4219-1-2026_0.pdf</t>
+          <t>4220-1-2026_0.pdf</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -10318,15 +10314,15 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>4219-1/2026.0</t>
+          <t>4220-1/2026.0</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_JUSANTE_4219-2026.pdf</t>
+          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AR_LAGOA-07_4220-2026.pdf</t>
         </is>
       </c>
     </row>
@@ -10338,7 +10334,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>4218-1-2026_0.pdf</t>
+          <t>4219-1-2026_0.pdf</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -10348,7 +10344,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>4218-1/2026.0</t>
+          <t>4219-1/2026.0</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
@@ -10356,12 +10352,42 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
+          <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_JUSANTE_4219-2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-20 14:48:36</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>4218-1-2026_0.pdf</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Processado</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>4218-1/2026.0</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
           <t>02_PROCESSADOS\2026\2026-09\2026-09-30_AB_REPRESA-1_4218-2026.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F11"/>
+  <autoFilter ref="A1:F12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>